<commit_message>
Fetch HKEX option quotes without Futu
</commit_message>
<xml_diff>
--- a/Trade Tracker.xlsx
+++ b/Trade Tracker.xlsx
@@ -17,8 +17,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="yyyy/m/d"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -63,12 +64,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -783,8 +785,8 @@
       <c r="B4" s="2" t="n">
         <v>46127</v>
       </c>
-      <c r="C4" s="2" t="n">
-        <v>46171</v>
+      <c r="C4" s="3" t="n">
+        <v>46170</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -858,8 +860,8 @@
       <c r="B5" s="2" t="n">
         <v>46132</v>
       </c>
-      <c r="C5" s="2" t="n">
-        <v>46171</v>
+      <c r="C5" s="3" t="n">
+        <v>46170</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -1427,7 +1429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U2"/>
+  <dimension ref="A1:U1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1560,7 +1562,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>